<commit_message>
adição do base do maps e da pasta utils e seu updt.
</commit_message>
<xml_diff>
--- a/docs/municipality.xlsx
+++ b/docs/municipality.xlsx
@@ -15,14 +15,14 @@
   <calcPr/>
   <extLst>
     <ext uri="GoogleSheetsCustomDataVersion2">
-      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="2m2nGdEubb6dVvHQIkoc3pxK+YWBiuvps1B92PHU6mA="/>
+      <go:sheetsCustomData xmlns:go="http://customooxmlschemas.google.com/" r:id="rId9" roundtripDataChecksum="IN4g8tlanN6uhQN0pg1SmMfqANjeChSt4sUQzUGta6U="/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="949" uniqueCount="301">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="950" uniqueCount="302">
   <si>
     <t>locality</t>
   </si>
@@ -838,6 +838,9 @@
   </si>
   <si>
     <t>USO E COBERTURA</t>
+  </si>
+  <si>
+    <t>MAPBIOMAS</t>
   </si>
   <si>
     <t>NM_MUN</t>
@@ -935,7 +938,7 @@
     <numFmt numFmtId="164" formatCode="0.000"/>
     <numFmt numFmtId="165" formatCode="0.0"/>
   </numFmts>
-  <fonts count="7">
+  <fonts count="10">
     <font>
       <sz val="10.0"/>
       <color rgb="FF000000"/>
@@ -959,8 +962,25 @@
       <name val="Arial"/>
     </font>
     <font>
+      <sz val="11.0"/>
+      <color rgb="FF000000"/>
+      <name val="&quot;Aptos Narrow&quot;"/>
+    </font>
+    <font>
       <color theme="1"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12.0"/>
+      <color theme="1"/>
+      <name val="Quicksand"/>
+    </font>
+    <font>
+      <sz val="8.0"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11.0"/>
@@ -973,7 +993,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -984,12 +1004,6 @@
       <patternFill patternType="solid">
         <fgColor theme="0"/>
         <bgColor theme="0"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFFF2CC"/>
       </patternFill>
     </fill>
     <fill>
@@ -1026,6 +1040,9 @@
     <xf borderId="0" fillId="0" fontId="3" numFmtId="1" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf borderId="0" fillId="0" fontId="4" numFmtId="1" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+    </xf>
     <xf borderId="0" fillId="0" fontId="3" numFmtId="1" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
@@ -1035,42 +1052,39 @@
     <xf borderId="0" fillId="2" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
-    </xf>
     <xf borderId="0" fillId="3" fontId="3" numFmtId="1" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="3" fontId="3" numFmtId="165" xfId="0" applyFont="1" applyNumberFormat="1"/>
-    <xf borderId="0" fillId="4" fontId="3" numFmtId="1" xfId="0" applyFill="1" applyFont="1" applyNumberFormat="1"/>
+    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="7" numFmtId="0" xfId="0" applyFont="1"/>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="8" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="left" readingOrder="0"/>
     </xf>
     <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyFont="1"/>
-    <xf borderId="0" fillId="5" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="2" numFmtId="0" xfId="0" applyFill="1" applyFont="1"/>
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment horizontal="right" readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="6" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="9" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="0" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
-    <xf borderId="0" fillId="5" fontId="4" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
+    <xf borderId="0" fillId="4" fontId="5" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment vertical="bottom"/>
     </xf>
   </cellXfs>
@@ -1304,7 +1318,7 @@
   <cols>
     <col customWidth="1" min="1" max="1" width="15.0"/>
     <col customWidth="1" min="2" max="2" width="13.13"/>
-    <col customWidth="1" min="3" max="3" width="19.25"/>
+    <col customWidth="1" min="3" max="3" width="18.88"/>
     <col customWidth="1" min="4" max="4" width="9.0"/>
     <col customWidth="1" min="5" max="5" width="22.5"/>
     <col customWidth="1" min="6" max="6" width="7.5"/>
@@ -1326,7 +1340,7 @@
     <col customWidth="1" min="23" max="23" width="21.0"/>
     <col customWidth="1" min="24" max="24" width="22.38"/>
     <col customWidth="1" min="25" max="25" width="20.0"/>
-    <col customWidth="1" min="26" max="26" width="19.75"/>
+    <col customWidth="1" min="26" max="29" width="19.75"/>
   </cols>
   <sheetData>
     <row r="1" ht="12.0" customHeight="1">
@@ -1408,6 +1422,9 @@
       <c r="Z1" s="1" t="s">
         <v>25</v>
       </c>
+      <c r="AA1" s="1"/>
+      <c r="AB1" s="1"/>
+      <c r="AC1" s="1"/>
     </row>
     <row r="2" ht="12.0" customHeight="1">
       <c r="A2" s="2" t="s">
@@ -1480,6 +1497,9 @@
       <c r="Z2" s="5">
         <v>1276.0</v>
       </c>
+      <c r="AA2" s="5"/>
+      <c r="AB2" s="8"/>
+      <c r="AC2" s="5"/>
     </row>
     <row r="3" ht="12.0" customHeight="1">
       <c r="A3" s="2" t="s">
@@ -1524,7 +1544,9 @@
       <c r="N3" s="6">
         <v>12.7</v>
       </c>
-      <c r="O3" s="8"/>
+      <c r="O3" s="9">
+        <v>0.0</v>
+      </c>
       <c r="P3" s="5">
         <v>3.0</v>
       </c>
@@ -1554,6 +1576,9 @@
       <c r="Z3" s="5">
         <v>287.0</v>
       </c>
+      <c r="AA3" s="5"/>
+      <c r="AB3" s="8"/>
+      <c r="AC3" s="5"/>
     </row>
     <row r="4" ht="12.0" customHeight="1">
       <c r="A4" s="2" t="s">
@@ -1632,6 +1657,9 @@
       <c r="Z4" s="5">
         <v>514.0</v>
       </c>
+      <c r="AA4" s="5"/>
+      <c r="AB4" s="8"/>
+      <c r="AC4" s="5"/>
     </row>
     <row r="5" ht="12.0" customHeight="1">
       <c r="A5" s="2" t="s">
@@ -1708,6 +1736,9 @@
       <c r="Z5" s="5">
         <v>1289.0</v>
       </c>
+      <c r="AA5" s="5"/>
+      <c r="AB5" s="8"/>
+      <c r="AC5" s="5"/>
     </row>
     <row r="6" ht="12.0" customHeight="1">
       <c r="A6" s="2" t="s">
@@ -1788,6 +1819,9 @@
       <c r="Z6" s="5">
         <v>1705.0</v>
       </c>
+      <c r="AA6" s="5"/>
+      <c r="AB6" s="8"/>
+      <c r="AC6" s="5"/>
     </row>
     <row r="7" ht="12.0" customHeight="1">
       <c r="A7" s="2" t="s">
@@ -1832,7 +1866,9 @@
       <c r="N7" s="6">
         <v>41.5</v>
       </c>
-      <c r="O7" s="8"/>
+      <c r="O7" s="9">
+        <v>0.0</v>
+      </c>
       <c r="P7" s="5">
         <v>1.0</v>
       </c>
@@ -1858,6 +1894,9 @@
       <c r="Z7" s="5">
         <v>395.0</v>
       </c>
+      <c r="AA7" s="5"/>
+      <c r="AB7" s="8"/>
+      <c r="AC7" s="5"/>
     </row>
     <row r="8" ht="12.0" customHeight="1">
       <c r="A8" s="2" t="s">
@@ -1936,6 +1975,9 @@
       <c r="Z8" s="5">
         <v>658.0</v>
       </c>
+      <c r="AA8" s="5"/>
+      <c r="AB8" s="8"/>
+      <c r="AC8" s="5"/>
     </row>
     <row r="9" ht="12.0" customHeight="1">
       <c r="A9" s="2" t="s">
@@ -1980,7 +2022,9 @@
       <c r="N9" s="6">
         <v>18.8</v>
       </c>
-      <c r="O9" s="8"/>
+      <c r="O9" s="9">
+        <v>0.0</v>
+      </c>
       <c r="P9" s="5"/>
       <c r="Q9" s="5"/>
       <c r="R9" s="5"/>
@@ -2008,50 +2052,80 @@
       <c r="Z9" s="5">
         <v>217.0</v>
       </c>
-    </row>
-    <row r="10" ht="12.0" customHeight="1">
-      <c r="A10" s="9" t="s">
+      <c r="AA9" s="5"/>
+      <c r="AB9" s="8"/>
+      <c r="AC9" s="5"/>
+    </row>
+    <row r="10" ht="11.25" customHeight="1">
+      <c r="A10" s="10" t="s">
         <v>26</v>
       </c>
-      <c r="B10" s="10">
+      <c r="B10" s="11">
         <v>3522653.0</v>
       </c>
-      <c r="C10" s="11" t="s">
+      <c r="C10" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="D10" s="12">
+      <c r="D10" s="13">
         <v>350004.0</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="E10" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="F10" s="12">
+      <c r="F10" s="13">
         <v>3502.0</v>
       </c>
-      <c r="G10" s="11" t="s">
+      <c r="G10" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="H10" s="13">
+      <c r="H10" s="4">
         <v>406.478</v>
       </c>
-      <c r="I10" s="14"/>
-      <c r="J10" s="14"/>
-      <c r="K10" s="14"/>
-      <c r="L10" s="15"/>
-      <c r="M10" s="15"/>
-      <c r="N10" s="15"/>
-      <c r="O10" s="8"/>
+      <c r="I10" s="5">
+        <v>4338.0</v>
+      </c>
+      <c r="J10" s="5">
+        <v>2247.0</v>
+      </c>
+      <c r="K10" s="5">
+        <v>2091.0</v>
+      </c>
+      <c r="L10" s="6">
+        <v>93.1</v>
+      </c>
+      <c r="M10" s="6">
+        <v>34.4</v>
+      </c>
+      <c r="N10" s="6">
+        <v>10.7</v>
+      </c>
+      <c r="O10" s="7">
+        <v>0.0</v>
+      </c>
       <c r="P10" s="5"/>
       <c r="Q10" s="5"/>
       <c r="R10" s="5"/>
       <c r="S10" s="5"/>
       <c r="T10" s="5"/>
       <c r="U10" s="5"/>
-      <c r="V10" s="5"/>
-      <c r="W10" s="5"/>
-      <c r="X10" s="5"/>
-      <c r="Y10" s="5"/>
-      <c r="Z10" s="5"/>
+      <c r="V10" s="5">
+        <v>2.0</v>
+      </c>
+      <c r="W10" s="5">
+        <v>2174.0</v>
+      </c>
+      <c r="X10" s="5">
+        <v>0.0</v>
+      </c>
+      <c r="Y10" s="5">
+        <v>2018.0</v>
+      </c>
+      <c r="Z10" s="5">
+        <v>112.0</v>
+      </c>
+      <c r="AA10" s="5"/>
+      <c r="AB10" s="8"/>
+      <c r="AC10" s="5"/>
     </row>
     <row r="11" ht="12.0" customHeight="1">
       <c r="A11" s="2" t="s">
@@ -2126,6 +2200,9 @@
       <c r="Z11" s="5">
         <v>1126.0</v>
       </c>
+      <c r="AA11" s="5"/>
+      <c r="AB11" s="8"/>
+      <c r="AC11" s="5"/>
     </row>
     <row r="12" ht="12.0" customHeight="1">
       <c r="A12" s="2" t="s">
@@ -2204,6 +2281,9 @@
       <c r="Z12" s="5">
         <v>665.0</v>
       </c>
+      <c r="AA12" s="5"/>
+      <c r="AB12" s="8"/>
+      <c r="AC12" s="5"/>
     </row>
     <row r="13" ht="12.0" customHeight="1">
       <c r="A13" s="2" t="s">
@@ -2280,6 +2360,9 @@
       <c r="Z13" s="5">
         <v>1012.0</v>
       </c>
+      <c r="AA13" s="5"/>
+      <c r="AB13" s="8"/>
+      <c r="AC13" s="5"/>
     </row>
     <row r="14" ht="12.0" customHeight="1">
       <c r="A14" s="2" t="s">
@@ -2352,6 +2435,9 @@
       <c r="Z14" s="5">
         <v>1667.0</v>
       </c>
+      <c r="AA14" s="5"/>
+      <c r="AB14" s="8"/>
+      <c r="AC14" s="5"/>
     </row>
     <row r="15" ht="12.0" customHeight="1">
       <c r="A15" s="2" t="s">
@@ -2406,11 +2492,11 @@
       <c r="R15" s="5">
         <v>156.0</v>
       </c>
-      <c r="S15" s="16">
+      <c r="S15" s="14">
         <v>39.0</v>
       </c>
-      <c r="T15" s="16"/>
-      <c r="U15" s="16"/>
+      <c r="T15" s="14"/>
+      <c r="U15" s="14"/>
       <c r="V15" s="5">
         <v>197.0</v>
       </c>
@@ -2426,6 +2512,9 @@
       <c r="Z15" s="5">
         <v>1102.0</v>
       </c>
+      <c r="AA15" s="5"/>
+      <c r="AB15" s="8"/>
+      <c r="AC15" s="5"/>
     </row>
     <row r="16" ht="12.0" customHeight="1">
       <c r="A16" s="2" t="s">
@@ -2502,6 +2591,9 @@
       <c r="Z16" s="5">
         <v>1017.0</v>
       </c>
+      <c r="AA16" s="5"/>
+      <c r="AB16" s="8"/>
+      <c r="AC16" s="5"/>
     </row>
     <row r="17" ht="12.0" customHeight="1">
       <c r="A17" s="2" t="s">
@@ -2574,6 +2666,9 @@
       <c r="Z17" s="5">
         <v>688.0</v>
       </c>
+      <c r="AA17" s="5"/>
+      <c r="AB17" s="8"/>
+      <c r="AC17" s="5"/>
     </row>
     <row r="18" ht="12.0" customHeight="1">
       <c r="A18" s="2" t="s">
@@ -2618,7 +2713,9 @@
       <c r="N18" s="6">
         <v>83.4</v>
       </c>
-      <c r="O18" s="8"/>
+      <c r="O18" s="9">
+        <v>0.0</v>
+      </c>
       <c r="P18" s="5">
         <v>189.0</v>
       </c>
@@ -2650,6 +2747,9 @@
       <c r="Z18" s="5">
         <v>3091.0</v>
       </c>
+      <c r="AA18" s="5"/>
+      <c r="AB18" s="8"/>
+      <c r="AC18" s="5"/>
     </row>
     <row r="19" ht="12.0" customHeight="1">
       <c r="A19" s="2" t="s">
@@ -2694,7 +2794,9 @@
       <c r="N19" s="6">
         <v>9.2</v>
       </c>
-      <c r="O19" s="8"/>
+      <c r="O19" s="9">
+        <v>0.0</v>
+      </c>
       <c r="P19" s="5"/>
       <c r="Q19" s="5"/>
       <c r="R19" s="5"/>
@@ -2716,6 +2818,9 @@
       <c r="Z19" s="5">
         <v>138.0</v>
       </c>
+      <c r="AA19" s="5"/>
+      <c r="AB19" s="8"/>
+      <c r="AC19" s="5"/>
     </row>
     <row r="20" ht="12.0" customHeight="1">
       <c r="A20" s="2" t="s">
@@ -2760,7 +2865,9 @@
       <c r="N20" s="6">
         <v>26.7</v>
       </c>
-      <c r="O20" s="8"/>
+      <c r="O20" s="9">
+        <v>0.0</v>
+      </c>
       <c r="P20" s="5">
         <v>21.0</v>
       </c>
@@ -2786,6 +2893,9 @@
       <c r="Z20" s="5">
         <v>565.0</v>
       </c>
+      <c r="AA20" s="5"/>
+      <c r="AB20" s="8"/>
+      <c r="AC20" s="5"/>
     </row>
     <row r="21" ht="12.0" customHeight="1">
       <c r="A21" s="2" t="s">
@@ -2858,6 +2968,9 @@
       <c r="Z21" s="5">
         <v>123.0</v>
       </c>
+      <c r="AA21" s="5"/>
+      <c r="AB21" s="8"/>
+      <c r="AC21" s="5"/>
     </row>
     <row r="22" ht="12.0" customHeight="1">
       <c r="A22" s="2" t="s">
@@ -2902,7 +3015,9 @@
       <c r="N22" s="6">
         <v>86.8</v>
       </c>
-      <c r="O22" s="8"/>
+      <c r="O22" s="9">
+        <v>0.0</v>
+      </c>
       <c r="P22" s="5">
         <v>11.0</v>
       </c>
@@ -2928,6 +3043,9 @@
       <c r="Z22" s="5">
         <v>982.0</v>
       </c>
+      <c r="AA22" s="5"/>
+      <c r="AB22" s="8"/>
+      <c r="AC22" s="5"/>
     </row>
     <row r="23" ht="12.0" customHeight="1">
       <c r="A23" s="2" t="s">
@@ -3004,6 +3122,9 @@
       <c r="Z23" s="5">
         <v>708.0</v>
       </c>
+      <c r="AA23" s="5"/>
+      <c r="AB23" s="8"/>
+      <c r="AC23" s="5"/>
     </row>
     <row r="24" ht="12.0" customHeight="1">
       <c r="A24" s="2" t="s">
@@ -3078,6 +3199,9 @@
       <c r="Z24" s="5">
         <v>457.0</v>
       </c>
+      <c r="AA24" s="5"/>
+      <c r="AB24" s="5"/>
+      <c r="AC24" s="5"/>
     </row>
     <row r="25" ht="12.0" customHeight="1">
       <c r="A25" s="2" t="s">
@@ -3122,7 +3246,9 @@
       <c r="N25" s="6">
         <v>267.0</v>
       </c>
-      <c r="O25" s="8"/>
+      <c r="O25" s="9">
+        <v>0.0</v>
+      </c>
       <c r="P25" s="5">
         <v>38.0</v>
       </c>
@@ -3148,6 +3274,9 @@
       <c r="Z25" s="5">
         <v>2007.0</v>
       </c>
+      <c r="AA25" s="5"/>
+      <c r="AB25" s="5"/>
+      <c r="AC25" s="5"/>
     </row>
     <row r="26" ht="12.0" customHeight="1">
       <c r="A26" s="2" t="s">
@@ -3192,7 +3321,9 @@
       <c r="N26" s="6">
         <v>14.7</v>
       </c>
-      <c r="O26" s="8"/>
+      <c r="O26" s="9">
+        <v>0.0</v>
+      </c>
       <c r="P26" s="5">
         <v>6.0</v>
       </c>
@@ -3218,6 +3349,9 @@
       <c r="Z26" s="5">
         <v>284.0</v>
       </c>
+      <c r="AA26" s="5"/>
+      <c r="AB26" s="5"/>
+      <c r="AC26" s="5"/>
     </row>
     <row r="27" ht="12.0" customHeight="1">
       <c r="A27" s="2" t="s">
@@ -3290,6 +3424,9 @@
       <c r="Z27" s="5">
         <v>260.0</v>
       </c>
+      <c r="AA27" s="5"/>
+      <c r="AB27" s="5"/>
+      <c r="AC27" s="5"/>
     </row>
     <row r="28" ht="12.0" customHeight="1">
       <c r="A28" s="2" t="s">
@@ -3362,6 +3499,9 @@
       <c r="Z28" s="5">
         <v>1034.0</v>
       </c>
+      <c r="AA28" s="5"/>
+      <c r="AB28" s="5"/>
+      <c r="AC28" s="5"/>
     </row>
     <row r="29" ht="12.0" customHeight="1">
       <c r="A29" s="2" t="s">
@@ -3434,6 +3574,9 @@
       <c r="Z29" s="5">
         <v>5629.0</v>
       </c>
+      <c r="AA29" s="5"/>
+      <c r="AB29" s="5"/>
+      <c r="AC29" s="5"/>
     </row>
     <row r="30" ht="12.0" customHeight="1">
       <c r="A30" s="2" t="s">
@@ -3506,6 +3649,9 @@
       <c r="Z30" s="5">
         <v>2145.0</v>
       </c>
+      <c r="AA30" s="5"/>
+      <c r="AB30" s="5"/>
+      <c r="AC30" s="5"/>
     </row>
     <row r="31" ht="12.0" customHeight="1">
       <c r="A31" s="2" t="s">
@@ -3578,6 +3724,9 @@
       <c r="Z31" s="5">
         <v>1559.0</v>
       </c>
+      <c r="AA31" s="5"/>
+      <c r="AB31" s="5"/>
+      <c r="AC31" s="5"/>
     </row>
     <row r="32" ht="12.0" customHeight="1">
       <c r="A32" s="2" t="s">
@@ -3622,7 +3771,9 @@
       <c r="N32" s="6">
         <v>93.2</v>
       </c>
-      <c r="O32" s="8"/>
+      <c r="O32" s="9">
+        <v>0.0</v>
+      </c>
       <c r="P32" s="5">
         <v>1.0</v>
       </c>
@@ -3648,6 +3799,9 @@
       <c r="Z32" s="5">
         <v>286.0</v>
       </c>
+      <c r="AA32" s="5"/>
+      <c r="AB32" s="5"/>
+      <c r="AC32" s="5"/>
     </row>
     <row r="33" ht="12.0" customHeight="1">
       <c r="A33" s="2" t="s">
@@ -3720,6 +3874,9 @@
       <c r="Z33" s="5">
         <v>5159.0</v>
       </c>
+      <c r="AA33" s="5"/>
+      <c r="AB33" s="5"/>
+      <c r="AC33" s="5"/>
     </row>
     <row r="34" ht="12.0" customHeight="1">
       <c r="A34" s="2" t="s">
@@ -3792,6 +3949,9 @@
       <c r="Z34" s="5">
         <v>664.0</v>
       </c>
+      <c r="AA34" s="5"/>
+      <c r="AB34" s="5"/>
+      <c r="AC34" s="5"/>
     </row>
     <row r="35" ht="12.0" customHeight="1">
       <c r="A35" s="2" t="s">
@@ -3864,6 +4024,9 @@
       <c r="Z35" s="5">
         <v>1979.0</v>
       </c>
+      <c r="AA35" s="5"/>
+      <c r="AB35" s="5"/>
+      <c r="AC35" s="5"/>
     </row>
     <row r="36" ht="12.0" customHeight="1">
       <c r="A36" s="2" t="s">
@@ -3940,6 +4103,9 @@
       <c r="Z36" s="5">
         <v>6925.0</v>
       </c>
+      <c r="AA36" s="5"/>
+      <c r="AB36" s="5"/>
+      <c r="AC36" s="5"/>
     </row>
     <row r="37" ht="12.0" customHeight="1">
       <c r="A37" s="2" t="s">
@@ -4012,6 +4178,9 @@
       <c r="Z37" s="5">
         <v>644.0</v>
       </c>
+      <c r="AA37" s="5"/>
+      <c r="AB37" s="5"/>
+      <c r="AC37" s="5"/>
     </row>
     <row r="38" ht="12.0" customHeight="1">
       <c r="A38" s="2" t="s">
@@ -4084,6 +4253,9 @@
       <c r="Z38" s="5">
         <v>14861.0</v>
       </c>
+      <c r="AA38" s="5"/>
+      <c r="AB38" s="5"/>
+      <c r="AC38" s="5"/>
     </row>
     <row r="39" ht="12.0" customHeight="1">
       <c r="A39" s="2" t="s">
@@ -4156,6 +4328,9 @@
       <c r="Z39" s="5">
         <v>286.0</v>
       </c>
+      <c r="AA39" s="5"/>
+      <c r="AB39" s="5"/>
+      <c r="AC39" s="5"/>
     </row>
     <row r="40" ht="12.0" customHeight="1">
       <c r="A40" s="2" t="s">
@@ -4228,6 +4403,9 @@
       <c r="Z40" s="5">
         <v>447.0</v>
       </c>
+      <c r="AA40" s="5"/>
+      <c r="AB40" s="5"/>
+      <c r="AC40" s="5"/>
     </row>
     <row r="41" ht="12.0" customHeight="1">
       <c r="A41" s="2" t="s">
@@ -4272,7 +4450,9 @@
       <c r="N41" s="6">
         <v>19.9</v>
       </c>
-      <c r="O41" s="8"/>
+      <c r="O41" s="9">
+        <v>0.0</v>
+      </c>
       <c r="P41" s="5">
         <v>3.0</v>
       </c>
@@ -4298,6 +4478,9 @@
       <c r="Z41" s="5">
         <v>180.0</v>
       </c>
+      <c r="AA41" s="5"/>
+      <c r="AB41" s="5"/>
+      <c r="AC41" s="5"/>
     </row>
     <row r="42" ht="12.0" customHeight="1">
       <c r="A42" s="2" t="s">
@@ -4370,6 +4553,9 @@
       <c r="Z42" s="5">
         <v>397.0</v>
       </c>
+      <c r="AA42" s="5"/>
+      <c r="AB42" s="5"/>
+      <c r="AC42" s="5"/>
     </row>
     <row r="43" ht="12.0" customHeight="1">
       <c r="A43" s="2" t="s">
@@ -4442,6 +4628,9 @@
       <c r="Z43" s="5">
         <v>5831.0</v>
       </c>
+      <c r="AA43" s="5"/>
+      <c r="AB43" s="5"/>
+      <c r="AC43" s="5"/>
     </row>
     <row r="44" ht="12.0" customHeight="1">
       <c r="A44" s="2" t="s">
@@ -4514,6 +4703,9 @@
       <c r="Z44" s="5">
         <v>248.0</v>
       </c>
+      <c r="AA44" s="5"/>
+      <c r="AB44" s="5"/>
+      <c r="AC44" s="5"/>
     </row>
     <row r="45" ht="12.0" customHeight="1">
       <c r="A45" s="2" t="s">
@@ -4586,6 +4778,9 @@
       <c r="Z45" s="5">
         <v>253.0</v>
       </c>
+      <c r="AA45" s="5"/>
+      <c r="AB45" s="5"/>
+      <c r="AC45" s="5"/>
     </row>
     <row r="46" ht="12.0" customHeight="1">
       <c r="A46" s="2" t="s">
@@ -4658,6 +4853,9 @@
       <c r="Z46" s="5">
         <v>882.0</v>
       </c>
+      <c r="AA46" s="5"/>
+      <c r="AB46" s="5"/>
+      <c r="AC46" s="5"/>
     </row>
     <row r="47" ht="12.0" customHeight="1">
       <c r="A47" s="2" t="s">
@@ -4730,6 +4928,9 @@
       <c r="Z47" s="5">
         <v>610.0</v>
       </c>
+      <c r="AA47" s="5"/>
+      <c r="AB47" s="5"/>
+      <c r="AC47" s="5"/>
     </row>
     <row r="48" ht="12.0" customHeight="1">
       <c r="A48" s="2" t="s">
@@ -4802,6 +5003,9 @@
       <c r="Z48" s="5">
         <v>10656.0</v>
       </c>
+      <c r="AA48" s="5"/>
+      <c r="AB48" s="5"/>
+      <c r="AC48" s="5"/>
     </row>
     <row r="49" ht="12.0" customHeight="1">
       <c r="A49" s="2" t="s">
@@ -4874,6 +5078,9 @@
       <c r="Z49" s="5">
         <v>942.0</v>
       </c>
+      <c r="AA49" s="5"/>
+      <c r="AB49" s="5"/>
+      <c r="AC49" s="5"/>
     </row>
     <row r="50" ht="12.0" customHeight="1">
       <c r="A50" s="2" t="s">
@@ -4946,6 +5153,9 @@
       <c r="Z50" s="5">
         <v>1257.0</v>
       </c>
+      <c r="AA50" s="5"/>
+      <c r="AB50" s="5"/>
+      <c r="AC50" s="5"/>
     </row>
     <row r="51" ht="12.0" customHeight="1">
       <c r="A51" s="2" t="s">
@@ -4990,7 +5200,9 @@
       <c r="N51" s="6">
         <v>457.9</v>
       </c>
-      <c r="O51" s="8"/>
+      <c r="O51" s="9">
+        <v>0.0</v>
+      </c>
       <c r="P51" s="5">
         <v>11.0</v>
       </c>
@@ -5016,6 +5228,9 @@
       <c r="Z51" s="5">
         <v>1347.0</v>
       </c>
+      <c r="AA51" s="5"/>
+      <c r="AB51" s="5"/>
+      <c r="AC51" s="5"/>
     </row>
     <row r="52" ht="12.0" customHeight="1">
       <c r="A52" s="2" t="s">
@@ -5088,6 +5303,9 @@
       <c r="Z52" s="5">
         <v>637.0</v>
       </c>
+      <c r="AA52" s="5"/>
+      <c r="AB52" s="5"/>
+      <c r="AC52" s="5"/>
     </row>
     <row r="53" ht="12.0" customHeight="1">
       <c r="A53" s="2" t="s">
@@ -5160,6 +5378,9 @@
       <c r="Z53" s="5">
         <v>178.0</v>
       </c>
+      <c r="AA53" s="5"/>
+      <c r="AB53" s="5"/>
+      <c r="AC53" s="5"/>
     </row>
     <row r="54" ht="12.0" customHeight="1">
       <c r="A54" s="2" t="s">
@@ -5204,7 +5425,9 @@
       <c r="N54" s="6">
         <v>83.9</v>
       </c>
-      <c r="O54" s="8"/>
+      <c r="O54" s="9">
+        <v>0.0</v>
+      </c>
       <c r="P54" s="5">
         <v>6.0</v>
       </c>
@@ -5230,6 +5453,9 @@
       <c r="Z54" s="5">
         <v>572.0</v>
       </c>
+      <c r="AA54" s="5"/>
+      <c r="AB54" s="5"/>
+      <c r="AC54" s="5"/>
     </row>
     <row r="55" ht="12.0" customHeight="1">
       <c r="A55" s="2" t="s">
@@ -5274,7 +5500,9 @@
       <c r="N55" s="6">
         <v>35.6</v>
       </c>
-      <c r="O55" s="8"/>
+      <c r="O55" s="9">
+        <v>0.0</v>
+      </c>
       <c r="P55" s="5">
         <v>4.0</v>
       </c>
@@ -5300,6 +5528,9 @@
       <c r="Z55" s="5">
         <v>395.0</v>
       </c>
+      <c r="AA55" s="5"/>
+      <c r="AB55" s="5"/>
+      <c r="AC55" s="5"/>
     </row>
     <row r="56" ht="12.0" customHeight="1">
       <c r="A56" s="2" t="s">
@@ -5372,6 +5603,9 @@
       <c r="Z56" s="5">
         <v>737.0</v>
       </c>
+      <c r="AA56" s="5"/>
+      <c r="AB56" s="5"/>
+      <c r="AC56" s="5"/>
     </row>
     <row r="57" ht="12.0" customHeight="1">
       <c r="A57" s="2" t="s">
@@ -5444,6 +5678,9 @@
       <c r="Z57" s="5">
         <v>3117.0</v>
       </c>
+      <c r="AA57" s="5"/>
+      <c r="AB57" s="5"/>
+      <c r="AC57" s="5"/>
     </row>
     <row r="58" ht="12.0" customHeight="1">
       <c r="A58" s="2" t="s">
@@ -5516,6 +5753,9 @@
       <c r="Z58" s="5">
         <v>157.0</v>
       </c>
+      <c r="AA58" s="5"/>
+      <c r="AB58" s="5"/>
+      <c r="AC58" s="5"/>
     </row>
     <row r="59" ht="12.0" customHeight="1">
       <c r="A59" s="2" t="s">
@@ -5592,6 +5832,9 @@
       <c r="Z59" s="5">
         <v>279.0</v>
       </c>
+      <c r="AA59" s="5"/>
+      <c r="AB59" s="5"/>
+      <c r="AC59" s="5"/>
     </row>
     <row r="60" ht="12.0" customHeight="1">
       <c r="A60" s="2" t="s">
@@ -5664,6 +5907,9 @@
       <c r="Z60" s="5">
         <v>198.0</v>
       </c>
+      <c r="AA60" s="5"/>
+      <c r="AB60" s="5"/>
+      <c r="AC60" s="5"/>
     </row>
     <row r="61" ht="12.0" customHeight="1">
       <c r="A61" s="2" t="s">
@@ -5736,6 +5982,9 @@
       <c r="Z61" s="5">
         <v>43136.0</v>
       </c>
+      <c r="AA61" s="5"/>
+      <c r="AB61" s="5"/>
+      <c r="AC61" s="5"/>
     </row>
     <row r="62" ht="12.0" customHeight="1">
       <c r="A62" s="2" t="s">
@@ -5808,6 +6057,9 @@
       <c r="Z62" s="5">
         <v>297.0</v>
       </c>
+      <c r="AA62" s="5"/>
+      <c r="AB62" s="5"/>
+      <c r="AC62" s="5"/>
     </row>
     <row r="63" ht="12.0" customHeight="1">
       <c r="A63" s="2" t="s">
@@ -5880,6 +6132,9 @@
       <c r="Z63" s="5">
         <v>351.0</v>
       </c>
+      <c r="AA63" s="5"/>
+      <c r="AB63" s="5"/>
+      <c r="AC63" s="5"/>
     </row>
     <row r="64" ht="12.0" customHeight="1">
       <c r="A64" s="2" t="s">
@@ -5952,6 +6207,9 @@
       <c r="Z64" s="5">
         <v>15384.0</v>
       </c>
+      <c r="AA64" s="5"/>
+      <c r="AB64" s="5"/>
+      <c r="AC64" s="5"/>
     </row>
     <row r="65" ht="12.0" customHeight="1">
       <c r="A65" s="2" t="s">
@@ -6024,6 +6282,9 @@
       <c r="Z65" s="5">
         <v>2682.0</v>
       </c>
+      <c r="AA65" s="5"/>
+      <c r="AB65" s="5"/>
+      <c r="AC65" s="5"/>
     </row>
     <row r="66" ht="12.0" customHeight="1">
       <c r="A66" s="2" t="s">
@@ -6102,6 +6363,9 @@
       <c r="Z66" s="5">
         <v>760.0</v>
       </c>
+      <c r="AA66" s="5"/>
+      <c r="AB66" s="5"/>
+      <c r="AC66" s="5"/>
     </row>
     <row r="67" ht="12.0" customHeight="1">
       <c r="A67" s="2" t="s">
@@ -6180,6 +6444,9 @@
       <c r="Z67" s="5">
         <v>1428.0</v>
       </c>
+      <c r="AA67" s="5"/>
+      <c r="AB67" s="5"/>
+      <c r="AC67" s="5"/>
     </row>
     <row r="68" ht="12.0" customHeight="1">
       <c r="A68" s="2" t="s">
@@ -6252,6 +6519,9 @@
       <c r="Z68" s="5">
         <v>867.0</v>
       </c>
+      <c r="AA68" s="5"/>
+      <c r="AB68" s="5"/>
+      <c r="AC68" s="5"/>
     </row>
     <row r="69" ht="12.0" customHeight="1">
       <c r="A69" s="2" t="s">
@@ -6324,6 +6594,9 @@
       <c r="Z69" s="5">
         <v>9775.0</v>
       </c>
+      <c r="AA69" s="5"/>
+      <c r="AB69" s="5"/>
+      <c r="AC69" s="5"/>
     </row>
     <row r="70" ht="12.0" customHeight="1">
       <c r="A70" s="2" t="s">
@@ -6396,6 +6669,9 @@
       <c r="Z70" s="5">
         <v>2641.0</v>
       </c>
+      <c r="AA70" s="5"/>
+      <c r="AB70" s="5"/>
+      <c r="AC70" s="5"/>
     </row>
     <row r="71" ht="12.0" customHeight="1">
       <c r="A71" s="2" t="s">
@@ -6470,6 +6746,9 @@
       <c r="Z71" s="5">
         <v>7492.0</v>
       </c>
+      <c r="AA71" s="5"/>
+      <c r="AB71" s="5"/>
+      <c r="AC71" s="5"/>
     </row>
     <row r="72" ht="12.0" customHeight="1">
       <c r="A72" s="2" t="s">
@@ -6550,6 +6829,9 @@
       <c r="Z72" s="5">
         <v>7364.0</v>
       </c>
+      <c r="AA72" s="5"/>
+      <c r="AB72" s="5"/>
+      <c r="AC72" s="5"/>
     </row>
     <row r="73" ht="12.0" customHeight="1"/>
     <row r="74" ht="12.0" customHeight="1"/>
@@ -7495,468 +7777,470 @@
   </sheetPr>
   <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.0"/>
   <cols>
-    <col customWidth="1" min="1" max="1" width="22.63"/>
-    <col customWidth="1" min="2" max="2" width="10.88"/>
-    <col customWidth="1" min="3" max="3" width="58.0"/>
-    <col customWidth="1" min="4" max="26" width="8.63"/>
+    <col customWidth="1" min="1" max="1" width="20.88"/>
+    <col customWidth="1" min="2" max="2" width="13.38"/>
+    <col customWidth="1" min="3" max="3" width="56.0"/>
+    <col customWidth="1" min="4" max="4" width="7.0"/>
+    <col customWidth="1" min="5" max="5" width="7.5"/>
+    <col customWidth="1" min="6" max="26" width="8.63"/>
   </cols>
   <sheetData>
     <row r="1" ht="12.0" customHeight="1">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="15" t="s">
         <v>194</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="15" t="s">
         <v>195</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="15" t="s">
         <v>196</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="15" t="s">
         <v>197</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="15" t="s">
         <v>198</v>
       </c>
     </row>
-    <row r="2" ht="12.0" customHeight="1">
-      <c r="A2" s="9" t="s">
+    <row r="2">
+      <c r="A2" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="16" t="s">
         <v>199</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="C2" s="16" t="s">
         <v>200</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="16" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="3" ht="12.0" customHeight="1">
-      <c r="A3" s="9" t="s">
+    <row r="3">
+      <c r="A3" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="B3" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C3" s="2" t="s">
+      <c r="C3" s="16" t="s">
         <v>203</v>
       </c>
-      <c r="D3" s="2">
+      <c r="D3" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="E3" s="16" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="4" ht="12.0" customHeight="1">
-      <c r="A4" s="9" t="s">
+    <row r="4">
+      <c r="A4" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="2" t="s">
+      <c r="B4" s="16" t="s">
         <v>199</v>
       </c>
-      <c r="C4" s="2" t="s">
+      <c r="C4" s="16" t="s">
         <v>204</v>
       </c>
-      <c r="D4" s="2">
+      <c r="D4" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="16" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="5" ht="12.0" customHeight="1">
-      <c r="A5" s="9" t="s">
+    <row r="5">
+      <c r="A5" s="10" t="s">
         <v>205</v>
       </c>
-      <c r="B5" s="2" t="s">
+      <c r="B5" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C5" s="2" t="s">
+      <c r="C5" s="16" t="s">
         <v>206</v>
       </c>
-      <c r="D5" s="2">
+      <c r="D5" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E5" s="2" t="s">
+      <c r="E5" s="16" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="6" ht="12.0" customHeight="1">
-      <c r="A6" s="9" t="s">
+    <row r="6">
+      <c r="A6" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="16" t="s">
         <v>199</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="16" t="s">
         <v>207</v>
       </c>
-      <c r="D6" s="2">
+      <c r="D6" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="16" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="7" ht="12.0" customHeight="1">
-      <c r="A7" s="9" t="s">
+    <row r="7">
+      <c r="A7" s="10" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C7" s="2" t="s">
+      <c r="C7" s="16" t="s">
         <v>208</v>
       </c>
-      <c r="D7" s="2">
+      <c r="D7" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E7" s="2" t="s">
+      <c r="E7" s="16" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="8" ht="12.0" customHeight="1">
-      <c r="A8" s="9" t="s">
+    <row r="8">
+      <c r="A8" s="10" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="2" t="s">
+      <c r="B8" s="16" t="s">
         <v>199</v>
       </c>
-      <c r="C8" s="2" t="s">
+      <c r="C8" s="16" t="s">
         <v>204</v>
       </c>
-      <c r="D8" s="2">
+      <c r="D8" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="16" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="9" ht="12.0" customHeight="1">
-      <c r="A9" s="9" t="s">
+    <row r="9">
+      <c r="A9" s="10" t="s">
         <v>7</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="B9" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C9" s="2" t="s">
+      <c r="C9" s="16" t="s">
         <v>209</v>
       </c>
-      <c r="D9" s="2">
+      <c r="D9" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E9" s="2" t="s">
+      <c r="E9" s="16" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="10" ht="12.0" customHeight="1">
-      <c r="A10" s="9" t="s">
+    <row r="10">
+      <c r="A10" s="10" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="B10" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C10" s="2" t="s">
+      <c r="C10" s="16" t="s">
         <v>210</v>
       </c>
-      <c r="D10" s="2">
+      <c r="D10" s="16">
         <v>2023.0</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="16" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="11" ht="12.0" customHeight="1">
-      <c r="A11" s="9" t="s">
+    <row r="11">
+      <c r="A11" s="10" t="s">
         <v>212</v>
       </c>
-      <c r="B11" s="2" t="s">
+      <c r="B11" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C11" s="2" t="s">
+      <c r="C11" s="16" t="s">
         <v>213</v>
       </c>
-      <c r="D11" s="2">
+      <c r="D11" s="16">
         <v>2023.0</v>
       </c>
-      <c r="E11" s="2" t="s">
+      <c r="E11" s="16" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="12" ht="12.0" customHeight="1">
-      <c r="A12" s="9" t="s">
+    <row r="12">
+      <c r="A12" s="10" t="s">
         <v>214</v>
       </c>
-      <c r="B12" s="2" t="s">
+      <c r="B12" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C12" s="2" t="s">
+      <c r="C12" s="16" t="s">
         <v>213</v>
       </c>
-      <c r="D12" s="2">
+      <c r="D12" s="16">
         <v>2023.0</v>
       </c>
-      <c r="E12" s="2" t="s">
+      <c r="E12" s="16" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="13" ht="12.0" customHeight="1">
-      <c r="A13" s="9" t="s">
+    <row r="13">
+      <c r="A13" s="10" t="s">
         <v>215</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="B13" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="C13" s="16" t="s">
         <v>216</v>
       </c>
-      <c r="D13" s="2">
+      <c r="D13" s="16">
         <v>2023.0</v>
       </c>
-      <c r="E13" s="2" t="s">
+      <c r="E13" s="16" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="14" ht="12.0" customHeight="1">
-      <c r="A14" s="9" t="s">
+    <row r="14">
+      <c r="A14" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="B14" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="C14" s="16" t="s">
         <v>217</v>
       </c>
-      <c r="D14" s="2">
+      <c r="D14" s="16">
         <v>2023.0</v>
       </c>
-      <c r="E14" s="2" t="s">
+      <c r="E14" s="16" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="15" ht="12.0" customHeight="1">
-      <c r="A15" s="9" t="s">
+    <row r="15">
+      <c r="A15" s="10" t="s">
         <v>13</v>
       </c>
-      <c r="B15" s="2" t="s">
+      <c r="B15" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C15" s="2" t="s">
+      <c r="C15" s="16" t="s">
         <v>218</v>
       </c>
-      <c r="D15" s="2">
+      <c r="D15" s="16">
         <v>2023.0</v>
       </c>
-      <c r="E15" s="2" t="s">
+      <c r="E15" s="16" t="s">
         <v>211</v>
       </c>
     </row>
-    <row r="16" ht="12.0" customHeight="1">
-      <c r="A16" s="9" t="s">
+    <row r="16">
+      <c r="A16" s="10" t="s">
         <v>14</v>
       </c>
-      <c r="B16" s="2" t="s">
+      <c r="B16" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C16" s="2" t="s">
+      <c r="C16" s="16" t="s">
         <v>219</v>
       </c>
-      <c r="D16" s="2">
+      <c r="D16" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E16" s="2" t="s">
+      <c r="E16" s="16" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="17" ht="12.0" customHeight="1">
-      <c r="A17" s="9" t="s">
+    <row r="17">
+      <c r="A17" s="10" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="2" t="s">
+      <c r="B17" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="C17" s="16" t="s">
         <v>220</v>
       </c>
-      <c r="D17" s="2">
+      <c r="D17" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E17" s="2" t="s">
+      <c r="E17" s="16" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="18" ht="12.0" customHeight="1">
-      <c r="A18" s="9" t="s">
+    <row r="18">
+      <c r="A18" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="B18" s="2" t="s">
+      <c r="B18" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C18" s="2" t="s">
+      <c r="C18" s="16" t="s">
         <v>221</v>
       </c>
-      <c r="D18" s="2">
+      <c r="D18" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E18" s="2" t="s">
+      <c r="E18" s="16" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="19" ht="12.0" customHeight="1">
-      <c r="A19" s="9" t="s">
+    <row r="19">
+      <c r="A19" s="10" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="2" t="s">
+      <c r="B19" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C19" s="2" t="s">
+      <c r="C19" s="16" t="s">
         <v>222</v>
       </c>
-      <c r="D19" s="2">
+      <c r="D19" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E19" s="2" t="s">
+      <c r="E19" s="16" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="20" ht="12.0" customHeight="1">
-      <c r="A20" s="9" t="s">
+    <row r="20">
+      <c r="A20" s="10" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="B20" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="C20" s="16" t="s">
         <v>223</v>
       </c>
-      <c r="D20" s="2">
+      <c r="D20" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E20" s="2" t="s">
+      <c r="E20" s="16" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="21" ht="12.0" customHeight="1">
-      <c r="A21" s="9" t="s">
+    <row r="21">
+      <c r="A21" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="2" t="s">
+      <c r="B21" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C21" s="2" t="s">
+      <c r="C21" s="16" t="s">
         <v>224</v>
       </c>
-      <c r="D21" s="2">
+      <c r="D21" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E21" s="2" t="s">
+      <c r="E21" s="16" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="22" ht="12.0" customHeight="1">
-      <c r="A22" s="9" t="s">
+    <row r="22">
+      <c r="A22" s="10" t="s">
         <v>20</v>
       </c>
-      <c r="B22" s="2" t="s">
+      <c r="B22" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C22" s="2" t="s">
+      <c r="C22" s="16" t="s">
         <v>225</v>
       </c>
-      <c r="D22" s="2">
+      <c r="D22" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E22" s="2" t="s">
+      <c r="E22" s="16" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="23" ht="12.0" customHeight="1">
-      <c r="A23" s="9" t="s">
+    <row r="23">
+      <c r="A23" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="B23" s="2" t="s">
+      <c r="B23" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C23" s="2" t="s">
+      <c r="C23" s="16" t="s">
         <v>226</v>
       </c>
-      <c r="D23" s="2">
+      <c r="D23" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E23" s="2" t="s">
+      <c r="E23" s="16" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="24" ht="12.0" customHeight="1">
-      <c r="A24" s="9" t="s">
+    <row r="24">
+      <c r="A24" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="B24" s="2" t="s">
+      <c r="B24" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C24" s="2" t="s">
+      <c r="C24" s="16" t="s">
         <v>226</v>
       </c>
-      <c r="D24" s="2">
+      <c r="D24" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E24" s="2" t="s">
+      <c r="E24" s="16" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="25" ht="12.0" customHeight="1">
-      <c r="A25" s="9" t="s">
+    <row r="25">
+      <c r="A25" s="10" t="s">
         <v>23</v>
       </c>
-      <c r="B25" s="2" t="s">
+      <c r="B25" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C25" s="2" t="s">
+      <c r="C25" s="16" t="s">
         <v>226</v>
       </c>
-      <c r="D25" s="2">
+      <c r="D25" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E25" s="2" t="s">
+      <c r="E25" s="16" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="26" ht="12.0" customHeight="1">
-      <c r="A26" s="9" t="s">
+    <row r="26">
+      <c r="A26" s="10" t="s">
         <v>24</v>
       </c>
-      <c r="B26" s="2" t="s">
+      <c r="B26" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C26" s="2" t="s">
+      <c r="C26" s="16" t="s">
         <v>226</v>
       </c>
-      <c r="D26" s="2">
+      <c r="D26" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E26" s="2" t="s">
+      <c r="E26" s="16" t="s">
         <v>201</v>
       </c>
     </row>
-    <row r="27" ht="12.0" customHeight="1">
-      <c r="A27" s="9" t="s">
+    <row r="27">
+      <c r="A27" s="10" t="s">
         <v>25</v>
       </c>
-      <c r="B27" s="2" t="s">
+      <c r="B27" s="16" t="s">
         <v>202</v>
       </c>
-      <c r="C27" s="2" t="s">
+      <c r="C27" s="16" t="s">
         <v>226</v>
       </c>
-      <c r="D27" s="2">
+      <c r="D27" s="16">
         <v>2022.0</v>
       </c>
-      <c r="E27" s="2" t="s">
+      <c r="E27" s="16" t="s">
         <v>201</v>
       </c>
     </row>
@@ -7977,7 +8261,7 @@
       <c r="A31" s="17" t="s">
         <v>230</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C31" s="10" t="s">
         <v>231</v>
       </c>
     </row>
@@ -7985,7 +8269,7 @@
       <c r="A32" s="2" t="s">
         <v>232</v>
       </c>
-      <c r="B32" s="9" t="s">
+      <c r="B32" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -7993,7 +8277,7 @@
       <c r="A33" s="2" t="s">
         <v>234</v>
       </c>
-      <c r="B33" s="9" t="s">
+      <c r="B33" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -8001,7 +8285,7 @@
       <c r="A34" s="2" t="s">
         <v>235</v>
       </c>
-      <c r="B34" s="9" t="s">
+      <c r="B34" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -8009,7 +8293,7 @@
       <c r="A35" s="2" t="s">
         <v>236</v>
       </c>
-      <c r="B35" s="9" t="s">
+      <c r="B35" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -8017,7 +8301,7 @@
       <c r="A36" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="B36" s="9" t="s">
+      <c r="B36" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -8025,31 +8309,31 @@
       <c r="A37" s="2" t="s">
         <v>238</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="B37" s="10" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="38" ht="12.0" customHeight="1">
-      <c r="A38" s="9" t="s">
+      <c r="A38" s="10" t="s">
         <v>239</v>
       </c>
-      <c r="B38" s="9" t="s">
+      <c r="B38" s="10" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="39" ht="12.0" customHeight="1">
-      <c r="A39" s="9" t="s">
+      <c r="A39" s="10" t="s">
         <v>240</v>
       </c>
-      <c r="B39" s="9" t="s">
+      <c r="B39" s="10" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="40" ht="12.0" customHeight="1">
-      <c r="A40" s="9" t="s">
+      <c r="A40" s="10" t="s">
         <v>241</v>
       </c>
-      <c r="B40" s="9" t="s">
+      <c r="B40" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -8057,7 +8341,7 @@
       <c r="A41" s="17" t="s">
         <v>242</v>
       </c>
-      <c r="C41" s="9" t="s">
+      <c r="C41" s="10" t="s">
         <v>243</v>
       </c>
     </row>
@@ -8118,7 +8402,7 @@
       <c r="A49" s="2" t="s">
         <v>251</v>
       </c>
-      <c r="B49" s="9" t="s">
+      <c r="B49" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -8126,7 +8410,7 @@
       <c r="A50" s="2" t="s">
         <v>252</v>
       </c>
-      <c r="B50" s="9" t="s">
+      <c r="B50" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -8134,7 +8418,7 @@
       <c r="A51" s="2" t="s">
         <v>253</v>
       </c>
-      <c r="B51" s="9" t="s">
+      <c r="B51" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -8142,7 +8426,7 @@
       <c r="A52" s="2" t="s">
         <v>254</v>
       </c>
-      <c r="B52" s="9" t="s">
+      <c r="B52" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -8150,7 +8434,7 @@
       <c r="A53" s="2" t="s">
         <v>255</v>
       </c>
-      <c r="B53" s="9" t="s">
+      <c r="B53" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -8158,7 +8442,7 @@
       <c r="A54" s="2" t="s">
         <v>256</v>
       </c>
-      <c r="B54" s="9" t="s">
+      <c r="B54" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -8166,7 +8450,7 @@
       <c r="A55" s="2" t="s">
         <v>257</v>
       </c>
-      <c r="B55" s="9" t="s">
+      <c r="B55" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -8174,7 +8458,7 @@
       <c r="A56" s="2" t="s">
         <v>258</v>
       </c>
-      <c r="B56" s="9" t="s">
+      <c r="B56" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -8182,7 +8466,7 @@
       <c r="A57" s="2" t="s">
         <v>259</v>
       </c>
-      <c r="B57" s="9" t="s">
+      <c r="B57" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -8190,7 +8474,7 @@
       <c r="A58" s="2" t="s">
         <v>260</v>
       </c>
-      <c r="B58" s="9" t="s">
+      <c r="B58" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -8198,7 +8482,7 @@
       <c r="A59" s="2" t="s">
         <v>261</v>
       </c>
-      <c r="B59" s="9" t="s">
+      <c r="B59" s="10" t="s">
         <v>233</v>
       </c>
     </row>
@@ -8206,12 +8490,12 @@
       <c r="A60" s="2" t="s">
         <v>262</v>
       </c>
-      <c r="B60" s="9" t="s">
+      <c r="B60" s="10" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="61" ht="12.0" customHeight="1">
-      <c r="A61" s="9" t="s">
+      <c r="A61" s="10" t="s">
         <v>263</v>
       </c>
     </row>
@@ -8222,37 +8506,37 @@
       </c>
     </row>
     <row r="64" ht="12.0" customHeight="1">
-      <c r="A64" s="9" t="s">
+      <c r="A64" s="10" t="s">
         <v>265</v>
       </c>
-      <c r="B64" s="9" t="s">
+      <c r="B64" s="10" t="s">
         <v>233</v>
       </c>
     </row>
     <row r="65" ht="12.0" customHeight="1">
-      <c r="A65" s="9" t="s">
+      <c r="A65" s="10" t="s">
         <v>266</v>
       </c>
-      <c r="B65" s="9" t="s">
+      <c r="B65" s="10" t="s">
         <v>233</v>
       </c>
-      <c r="C65" s="9" t="s">
+      <c r="C65" s="10" t="s">
         <v>267</v>
       </c>
     </row>
     <row r="66" ht="12.0" customHeight="1">
-      <c r="A66" s="9" t="s">
+      <c r="A66" s="10" t="s">
         <v>268</v>
       </c>
-      <c r="C66" s="9" t="s">
+      <c r="C66" s="10" t="s">
         <v>269</v>
       </c>
     </row>
     <row r="67" ht="12.0" customHeight="1">
-      <c r="A67" s="9" t="s">
+      <c r="A67" s="10" t="s">
         <v>270</v>
       </c>
-      <c r="C67" s="9" t="s">
+      <c r="C67" s="10" t="s">
         <v>269</v>
       </c>
     </row>
@@ -8260,7 +8544,10 @@
       <c r="A68" s="17" t="s">
         <v>271</v>
       </c>
-      <c r="C68" s="9" t="s">
+      <c r="B68" s="10" t="s">
+        <v>272</v>
+      </c>
+      <c r="C68" s="10" t="s">
         <v>267</v>
       </c>
     </row>
@@ -9217,23 +9504,23 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="20" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>273</v>
+        <v>274</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>274</v>
+        <v>275</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="B2" s="9">
+      <c r="B2" s="10">
         <v>11.0</v>
       </c>
-      <c r="C2" s="9">
+      <c r="C2" s="10">
         <v>14.0</v>
       </c>
     </row>
@@ -9241,7 +9528,7 @@
       <c r="A3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="9">
+      <c r="B3" s="10">
         <v>11.0</v>
       </c>
     </row>
@@ -9249,7 +9536,7 @@
       <c r="A4" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="B4" s="9">
+      <c r="B4" s="10">
         <v>11.0</v>
       </c>
     </row>
@@ -9257,7 +9544,7 @@
       <c r="A5" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="B5" s="9">
+      <c r="B5" s="10">
         <v>11.0</v>
       </c>
     </row>
@@ -9265,7 +9552,7 @@
       <c r="A6" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="B6" s="9">
+      <c r="B6" s="10">
         <v>11.0</v>
       </c>
     </row>
@@ -9273,7 +9560,7 @@
       <c r="A7" s="21" t="s">
         <v>44</v>
       </c>
-      <c r="B7" s="9">
+      <c r="B7" s="10">
         <v>14.0</v>
       </c>
     </row>
@@ -9281,7 +9568,7 @@
       <c r="A8" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="B8" s="9">
+      <c r="B8" s="10">
         <v>11.0</v>
       </c>
     </row>
@@ -9289,15 +9576,15 @@
       <c r="A9" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="B9" s="9">
+      <c r="B9" s="10">
         <v>11.0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="12" t="s">
         <v>49</v>
       </c>
-      <c r="B10" s="9">
+      <c r="B10" s="10">
         <v>11.0</v>
       </c>
     </row>
@@ -9305,10 +9592,10 @@
       <c r="A11" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="B11" s="9">
+      <c r="B11" s="10">
         <v>11.0</v>
       </c>
-      <c r="C11" s="9">
+      <c r="C11" s="10">
         <v>7.0</v>
       </c>
     </row>
@@ -9316,7 +9603,7 @@
       <c r="A12" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="B12" s="9">
+      <c r="B12" s="10">
         <v>11.0</v>
       </c>
     </row>
@@ -9324,7 +9611,7 @@
       <c r="A13" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="B13" s="9">
+      <c r="B13" s="10">
         <v>11.0</v>
       </c>
     </row>
@@ -9332,7 +9619,7 @@
       <c r="A14" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="B14" s="9">
+      <c r="B14" s="10">
         <v>11.0</v>
       </c>
     </row>
@@ -9340,7 +9627,7 @@
       <c r="A15" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B15" s="9">
+      <c r="B15" s="10">
         <v>11.0</v>
       </c>
     </row>
@@ -9348,7 +9635,7 @@
       <c r="A16" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="B16" s="9">
+      <c r="B16" s="10">
         <v>11.0</v>
       </c>
     </row>
@@ -9356,7 +9643,7 @@
       <c r="A17" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="B17" s="9">
+      <c r="B17" s="10">
         <v>11.0</v>
       </c>
     </row>
@@ -9364,7 +9651,7 @@
       <c r="A18" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="10">
         <v>11.0</v>
       </c>
     </row>
@@ -9372,7 +9659,7 @@
       <c r="A19" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="B19" s="9">
+      <c r="B19" s="10">
         <v>11.0</v>
       </c>
     </row>
@@ -9380,7 +9667,7 @@
       <c r="A20" s="21" t="s">
         <v>73</v>
       </c>
-      <c r="B20" s="9">
+      <c r="B20" s="10">
         <v>14.0</v>
       </c>
     </row>
@@ -9388,7 +9675,7 @@
       <c r="A21" s="21" t="s">
         <v>75</v>
       </c>
-      <c r="B21" s="9">
+      <c r="B21" s="10">
         <v>14.0</v>
       </c>
     </row>
@@ -9396,7 +9683,7 @@
       <c r="A22" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="B22" s="9">
+      <c r="B22" s="10">
         <v>11.0</v>
       </c>
     </row>
@@ -9404,7 +9691,7 @@
       <c r="A23" s="2" t="s">
         <v>79</v>
       </c>
-      <c r="B23" s="9">
+      <c r="B23" s="10">
         <v>11.0</v>
       </c>
     </row>
@@ -9412,10 +9699,10 @@
       <c r="A24" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="B24" s="9">
+      <c r="B24" s="10">
         <v>11.0</v>
       </c>
-      <c r="C24" s="9">
+      <c r="C24" s="10">
         <v>14.0</v>
       </c>
     </row>
@@ -9423,7 +9710,7 @@
       <c r="A25" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="B25" s="9">
+      <c r="B25" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9431,7 +9718,7 @@
       <c r="A26" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="B26" s="9">
+      <c r="B26" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9439,7 +9726,7 @@
       <c r="A27" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="B27" s="9">
+      <c r="B27" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9447,7 +9734,7 @@
       <c r="A28" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="B28" s="9">
+      <c r="B28" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9455,7 +9742,7 @@
       <c r="A29" s="2" t="s">
         <v>99</v>
       </c>
-      <c r="B29" s="9">
+      <c r="B29" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9463,7 +9750,7 @@
       <c r="A30" s="2" t="s">
         <v>102</v>
       </c>
-      <c r="B30" s="9">
+      <c r="B30" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9471,7 +9758,7 @@
       <c r="A31" s="2" t="s">
         <v>104</v>
       </c>
-      <c r="B31" s="9">
+      <c r="B31" s="10">
         <v>1.0</v>
       </c>
     </row>
@@ -9479,7 +9766,7 @@
       <c r="A32" s="2" t="s">
         <v>108</v>
       </c>
-      <c r="B32" s="9">
+      <c r="B32" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9487,7 +9774,7 @@
       <c r="A33" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="B33" s="9">
+      <c r="B33" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9495,7 +9782,7 @@
       <c r="A34" s="2" t="s">
         <v>111</v>
       </c>
-      <c r="B34" s="9">
+      <c r="B34" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9503,7 +9790,7 @@
       <c r="A35" s="21" t="s">
         <v>113</v>
       </c>
-      <c r="B35" s="9">
+      <c r="B35" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9511,7 +9798,7 @@
       <c r="A36" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="B36" s="9">
+      <c r="B36" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9519,7 +9806,7 @@
       <c r="A37" s="2" t="s">
         <v>116</v>
       </c>
-      <c r="B37" s="9">
+      <c r="B37" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9527,7 +9814,7 @@
       <c r="A38" s="2" t="s">
         <v>118</v>
       </c>
-      <c r="B38" s="9">
+      <c r="B38" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9535,7 +9822,7 @@
       <c r="A39" s="2" t="s">
         <v>120</v>
       </c>
-      <c r="B39" s="9">
+      <c r="B39" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9543,7 +9830,7 @@
       <c r="A40" s="21" t="s">
         <v>122</v>
       </c>
-      <c r="B40" s="9">
+      <c r="B40" s="10">
         <v>5.0</v>
       </c>
     </row>
@@ -9551,7 +9838,7 @@
       <c r="A41" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B41" s="9">
+      <c r="B41" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9559,7 +9846,7 @@
       <c r="A42" s="2" t="s">
         <v>130</v>
       </c>
-      <c r="B42" s="9">
+      <c r="B42" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9567,7 +9854,7 @@
       <c r="A43" s="2" t="s">
         <v>132</v>
       </c>
-      <c r="B43" s="9">
+      <c r="B43" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9575,7 +9862,7 @@
       <c r="A44" s="2" t="s">
         <v>134</v>
       </c>
-      <c r="B44" s="9">
+      <c r="B44" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9583,7 +9870,7 @@
       <c r="A45" s="2" t="s">
         <v>136</v>
       </c>
-      <c r="B45" s="9">
+      <c r="B45" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9591,10 +9878,10 @@
       <c r="A46" s="21" t="s">
         <v>138</v>
       </c>
-      <c r="B46" s="9">
+      <c r="B46" s="10">
         <v>5.0</v>
       </c>
-      <c r="C46" s="9">
+      <c r="C46" s="10">
         <v>6.0</v>
       </c>
     </row>
@@ -9602,10 +9889,10 @@
       <c r="A47" s="2" t="s">
         <v>140</v>
       </c>
-      <c r="B47" s="9">
+      <c r="B47" s="10">
         <v>2.0</v>
       </c>
-      <c r="C47" s="9">
+      <c r="C47" s="10">
         <v>6.0</v>
       </c>
     </row>
@@ -9613,7 +9900,7 @@
       <c r="A48" s="2" t="s">
         <v>142</v>
       </c>
-      <c r="B48" s="9">
+      <c r="B48" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9621,7 +9908,7 @@
       <c r="A49" s="2" t="s">
         <v>144</v>
       </c>
-      <c r="B49" s="9">
+      <c r="B49" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9629,7 +9916,7 @@
       <c r="A50" s="21" t="s">
         <v>146</v>
       </c>
-      <c r="B50" s="9">
+      <c r="B50" s="10">
         <v>5.0</v>
       </c>
     </row>
@@ -9637,7 +9924,7 @@
       <c r="A51" s="2" t="s">
         <v>148</v>
       </c>
-      <c r="B51" s="9">
+      <c r="B51" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9645,7 +9932,7 @@
       <c r="A52" s="2" t="s">
         <v>150</v>
       </c>
-      <c r="B52" s="9">
+      <c r="B52" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9653,7 +9940,7 @@
       <c r="A53" s="2" t="s">
         <v>152</v>
       </c>
-      <c r="B53" s="9">
+      <c r="B53" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9661,7 +9948,7 @@
       <c r="A54" s="2" t="s">
         <v>154</v>
       </c>
-      <c r="B54" s="9">
+      <c r="B54" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9669,7 +9956,7 @@
       <c r="A55" s="21" t="s">
         <v>156</v>
       </c>
-      <c r="B55" s="9">
+      <c r="B55" s="10">
         <v>6.0</v>
       </c>
     </row>
@@ -9677,7 +9964,7 @@
       <c r="A56" s="2" t="s">
         <v>158</v>
       </c>
-      <c r="B56" s="9">
+      <c r="B56" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9685,7 +9972,7 @@
       <c r="A57" s="21" t="s">
         <v>160</v>
       </c>
-      <c r="B57" s="9">
+      <c r="B57" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9693,7 +9980,7 @@
       <c r="A58" s="2" t="s">
         <v>162</v>
       </c>
-      <c r="B58" s="9">
+      <c r="B58" s="10">
         <v>1.0</v>
       </c>
     </row>
@@ -9701,7 +9988,7 @@
       <c r="A59" s="2" t="s">
         <v>164</v>
       </c>
-      <c r="B59" s="9">
+      <c r="B59" s="10">
         <v>1.0</v>
       </c>
     </row>
@@ -9709,7 +9996,7 @@
       <c r="A60" s="2" t="s">
         <v>166</v>
       </c>
-      <c r="B60" s="9">
+      <c r="B60" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9717,7 +10004,7 @@
       <c r="A61" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="B61" s="9">
+      <c r="B61" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9725,7 +10012,7 @@
       <c r="A62" s="2" t="s">
         <v>169</v>
       </c>
-      <c r="B62" s="9">
+      <c r="B62" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9733,7 +10020,7 @@
       <c r="A63" s="2" t="s">
         <v>171</v>
       </c>
-      <c r="B63" s="9">
+      <c r="B63" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9741,7 +10028,7 @@
       <c r="A64" s="2" t="s">
         <v>173</v>
       </c>
-      <c r="B64" s="9">
+      <c r="B64" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9749,7 +10036,7 @@
       <c r="A65" s="2" t="s">
         <v>175</v>
       </c>
-      <c r="B65" s="9">
+      <c r="B65" s="10">
         <v>2.0</v>
       </c>
     </row>
@@ -9757,7 +10044,7 @@
       <c r="A66" s="2" t="s">
         <v>178</v>
       </c>
-      <c r="B66" s="9">
+      <c r="B66" s="10">
         <v>11.0</v>
       </c>
     </row>
@@ -9765,7 +10052,7 @@
       <c r="A67" s="2" t="s">
         <v>180</v>
       </c>
-      <c r="B67" s="9">
+      <c r="B67" s="10">
         <v>11.0</v>
       </c>
     </row>
@@ -9773,7 +10060,7 @@
       <c r="A68" s="2" t="s">
         <v>182</v>
       </c>
-      <c r="B68" s="9">
+      <c r="B68" s="10">
         <v>11.0</v>
       </c>
     </row>
@@ -9781,7 +10068,7 @@
       <c r="A69" s="2" t="s">
         <v>185</v>
       </c>
-      <c r="B69" s="9">
+      <c r="B69" s="10">
         <v>3.0</v>
       </c>
     </row>
@@ -9789,7 +10076,7 @@
       <c r="A70" s="2" t="s">
         <v>189</v>
       </c>
-      <c r="B70" s="9">
+      <c r="B70" s="10">
         <v>3.0</v>
       </c>
     </row>
@@ -9797,7 +10084,7 @@
       <c r="A71" s="2" t="s">
         <v>191</v>
       </c>
-      <c r="B71" s="9">
+      <c r="B71" s="10">
         <v>3.0</v>
       </c>
     </row>
@@ -9805,7 +10092,7 @@
       <c r="A72" s="2" t="s">
         <v>193</v>
       </c>
-      <c r="B72" s="9">
+      <c r="B72" s="10">
         <v>3.0</v>
       </c>
     </row>
@@ -9827,13 +10114,13 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="22" t="s">
-        <v>275</v>
+        <v>276</v>
       </c>
       <c r="B1" s="22" t="s">
-        <v>276</v>
+        <v>277</v>
       </c>
       <c r="C1" s="17" t="s">
-        <v>277</v>
+        <v>278</v>
       </c>
       <c r="D1" s="17" t="s">
         <v>2</v>
@@ -9843,26 +10130,26 @@
       <c r="A2" s="23">
         <v>1.0</v>
       </c>
-      <c r="B2" s="11" t="s">
-        <v>278</v>
-      </c>
-      <c r="D2" s="9" t="s">
+      <c r="B2" s="12" t="s">
         <v>279</v>
+      </c>
+      <c r="D2" s="10" t="s">
+        <v>280</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="23">
         <v>2.0</v>
       </c>
-      <c r="B3" s="11" t="s">
-        <v>280</v>
+      <c r="B3" s="12" t="s">
+        <v>281</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="23">
         <v>3.0</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="12" t="s">
         <v>183</v>
       </c>
     </row>
@@ -9870,152 +10157,152 @@
       <c r="A5" s="23">
         <v>4.0</v>
       </c>
-      <c r="B5" s="11" t="s">
-        <v>281</v>
+      <c r="B5" s="12" t="s">
+        <v>282</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="23">
         <v>5.0</v>
       </c>
-      <c r="B6" s="11" t="s">
-        <v>282</v>
+      <c r="B6" s="12" t="s">
+        <v>283</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="23">
         <v>6.0</v>
       </c>
-      <c r="B7" s="11" t="s">
-        <v>283</v>
+      <c r="B7" s="12" t="s">
+        <v>284</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="23">
         <v>7.0</v>
       </c>
-      <c r="B8" s="11" t="s">
-        <v>284</v>
+      <c r="B8" s="12" t="s">
+        <v>285</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="23">
         <v>8.0</v>
       </c>
-      <c r="B9" s="11" t="s">
-        <v>285</v>
+      <c r="B9" s="12" t="s">
+        <v>286</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="23">
         <v>9.0</v>
       </c>
-      <c r="B10" s="11" t="s">
-        <v>286</v>
+      <c r="B10" s="12" t="s">
+        <v>287</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="23">
         <v>10.0</v>
       </c>
-      <c r="B11" s="11" t="s">
-        <v>287</v>
+      <c r="B11" s="12" t="s">
+        <v>288</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="23">
         <v>11.0</v>
       </c>
-      <c r="B12" s="11" t="s">
-        <v>288</v>
+      <c r="B12" s="12" t="s">
+        <v>289</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="23">
         <v>12.0</v>
       </c>
-      <c r="B13" s="11" t="s">
-        <v>289</v>
+      <c r="B13" s="12" t="s">
+        <v>290</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="23">
         <v>13.0</v>
       </c>
-      <c r="B14" s="11" t="s">
-        <v>290</v>
+      <c r="B14" s="12" t="s">
+        <v>291</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="23">
         <v>14.0</v>
       </c>
-      <c r="B15" s="11" t="s">
-        <v>291</v>
+      <c r="B15" s="12" t="s">
+        <v>292</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="23">
         <v>15.0</v>
       </c>
-      <c r="B16" s="11" t="s">
-        <v>292</v>
+      <c r="B16" s="12" t="s">
+        <v>293</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="23">
         <v>16.0</v>
       </c>
-      <c r="B17" s="11" t="s">
-        <v>293</v>
+      <c r="B17" s="12" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="23">
         <v>17.0</v>
       </c>
-      <c r="B18" s="11" t="s">
-        <v>294</v>
+      <c r="B18" s="12" t="s">
+        <v>295</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="23">
         <v>18.0</v>
       </c>
-      <c r="B19" s="11" t="s">
-        <v>295</v>
+      <c r="B19" s="12" t="s">
+        <v>296</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="23">
         <v>19.0</v>
       </c>
-      <c r="B20" s="11" t="s">
-        <v>296</v>
+      <c r="B20" s="12" t="s">
+        <v>297</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="23">
         <v>20.0</v>
       </c>
-      <c r="B21" s="11" t="s">
-        <v>297</v>
+      <c r="B21" s="12" t="s">
+        <v>298</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="23">
         <v>21.0</v>
       </c>
-      <c r="B22" s="11" t="s">
-        <v>298</v>
+      <c r="B22" s="12" t="s">
+        <v>299</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="23">
         <v>22.0</v>
       </c>
-      <c r="B23" s="11" t="s">
-        <v>299</v>
+      <c r="B23" s="12" t="s">
+        <v>300</v>
       </c>
     </row>
   </sheetData>
@@ -10032,10 +10319,10 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="24" t="s">
-        <v>300</v>
+        <v>301</v>
       </c>
       <c r="B1" s="24" t="s">
-        <v>272</v>
+        <v>273</v>
       </c>
     </row>
     <row r="2">

</xml_diff>